<commit_message>
Zoho deals matched to the real All Deals by Stage report
The 04 template now takes the Zoho report pasted whole from A1: the title
rows are skipped, the stage group headings with their counts are read
and carried down to the deals under them, and the columns are the
report's own, with CTS DEPARTMENT mapped to portal departments on a
Departments tab and Opportunity Number kept as the job number. Build
reports won, lost and open counts and any Zoho department with no portal
home. The pipeline layer weights open deals by stage with the report's
real stage names, counts won deals as confirmed in their closing month by
default, and never counts a deal whose job number an order or quote
already carries. Checked against the real export: 663 deals, 483 won,
117 lost, 63 open, 12 Multi-Service left for the Departments tab.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016pDBrZS7dfZTTsSsTFUkBU
</commit_message>
<xml_diff>
--- a/portal/templates/08 Config.xlsx
+++ b/portal/templates/08 Config.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -768,15 +768,28 @@
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
+          <t>Portal link</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr"/>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Where people open the portal: the SharePoint link to CTS Business Intelligence Portal.html, or the synced folder path. Goes in every email</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
           <t>Portal version</t>
         </is>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>2.0.0</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr"/>
+      <c r="C11" s="9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4640,7 +4653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5413,7 +5426,7 @@
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>Charts</t>
+          <t>Trends</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
@@ -5466,12 +5479,12 @@
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>loaders</t>
+          <t>build</t>
         </is>
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>Data Loaders</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
@@ -5491,12 +5504,12 @@
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>build</t>
+          <t>distribution</t>
         </is>
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Distribution</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
@@ -5516,12 +5529,12 @@
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>distribution</t>
+          <t>config</t>
         </is>
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>Distribution</t>
+          <t>Config &amp; Variables</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
@@ -5541,12 +5554,12 @@
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>config</t>
+          <t>access</t>
         </is>
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>Config &amp; Variables</t>
+          <t>Access Control</t>
         </is>
       </c>
       <c r="C30" s="9" t="inlineStr">
@@ -5554,11 +5567,7 @@
           <t>Always</t>
         </is>
       </c>
-      <c r="D30" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="D30" s="11" t="inlineStr"/>
       <c r="E30" s="11" t="inlineStr"/>
       <c r="F30" s="11" t="inlineStr"/>
       <c r="G30" s="11" t="inlineStr"/>
@@ -5566,12 +5575,12 @@
     <row r="31">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>access</t>
+          <t>about</t>
         </is>
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>Access Control</t>
+          <t>About</t>
         </is>
       </c>
       <c r="C31" s="9" t="inlineStr">
@@ -5579,43 +5588,22 @@
           <t>Always</t>
         </is>
       </c>
-      <c r="D31" s="11" t="inlineStr"/>
-      <c r="E31" s="11" t="inlineStr"/>
-      <c r="F31" s="11" t="inlineStr"/>
-      <c r="G31" s="11" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="9" t="inlineStr">
-        <is>
-          <t>about</t>
-        </is>
-      </c>
-      <c r="B32" s="9" t="inlineStr">
-        <is>
-          <t>About</t>
-        </is>
-      </c>
-      <c r="C32" s="9" t="inlineStr">
-        <is>
-          <t>Always</t>
-        </is>
-      </c>
-      <c r="D32" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E32" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F32" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G32" s="11" t="inlineStr">
+      <c r="D31" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E31" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F31" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G31" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>

</xml_diff>